<commit_message>
fix(quests): reconcile September history and preserve planning work
</commit_message>
<xml_diff>
--- a/outputs/dd-silver-plan-2026-09-05/DD7-silver-plan-final.xlsx
+++ b/outputs/dd-silver-plan-2026-09-05/DD7-silver-plan-final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liqui\Documents\farmrpg-tools\outputs\dd-silver-plan-2026-09-05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9144705-6217-440C-8EDB-0E15889B813F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBAE5E9-9DEB-4535-BFB9-087E15E37DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>Silver on hand</t>
   </si>
   <si>
-    <t>3.042T</t>
-  </si>
-  <si>
     <t>Bank</t>
   </si>
   <si>
@@ -195,6 +192,9 @@
   </si>
   <si>
     <t>Enter value / planned sell price</t>
+  </si>
+  <si>
+    <t>3.852t</t>
   </si>
 </sst>
 </file>
@@ -796,7 +796,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>5</v>
@@ -829,11 +829,11 @@
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="50" t="s">
-        <v>9</v>
+        <v>53</v>
       </c>
       <c r="D8" s="51">
         <f>IF(C8="","",LEFT(TRIM(C8),LEN(TRIM(C8))-1)*IF(RIGHT(UPPER(TRIM(C8)),1)="T",1000000000000,IF(RIGHT(UPPER(TRIM(C8)),1)="B",1000000000,IF(RIGHT(UPPER(TRIM(C8)),1)="M",1000000,1))))</f>
-        <v>3042000000000</v>
+        <v>3852000000000</v>
       </c>
       <c r="E8" s="20"/>
       <c r="F8" s="22"/>
@@ -842,11 +842,11 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A9" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="51">
         <f>IF(C9="","",LEFT(TRIM(C9),LEN(TRIM(C9))-1)*IF(RIGHT(UPPER(TRIM(C9)),1)="T",1000000000000,IF(RIGHT(UPPER(TRIM(C9)),1)="B",1000000000,IF(RIGHT(UPPER(TRIM(C9)),1)="M",1000000,1))))</f>
@@ -859,17 +859,17 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A10" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="21">
-        <v>3612</v>
+        <v>2500</v>
       </c>
       <c r="C10" s="41">
         <v>190000000</v>
       </c>
       <c r="D10" s="42">
         <f>B10*C10</f>
-        <v>686280000000</v>
+        <v>475000000000</v>
       </c>
       <c r="E10" s="20"/>
       <c r="F10" s="22"/>
@@ -878,17 +878,17 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A11" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="21">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="C11" s="41">
         <v>600000000</v>
       </c>
       <c r="D11" s="42">
         <f>B11*C11</f>
-        <v>69000000000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="20"/>
       <c r="F11" s="22"/>
@@ -897,13 +897,13 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A12" s="33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="34"/>
       <c r="C12" s="34"/>
       <c r="D12" s="43">
         <f>SUM(D8:D11)</f>
-        <v>4397580000000</v>
+        <v>4927300000000</v>
       </c>
       <c r="E12" s="20"/>
       <c r="F12" s="22"/>
@@ -912,13 +912,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A13" s="14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="23"/>
       <c r="C13" s="23"/>
       <c r="D13" s="44">
         <f>MAX(0,D7-D12)</f>
-        <v>602420000000</v>
+        <v>72700000000</v>
       </c>
       <c r="E13" s="20"/>
       <c r="F13" s="22"/>
@@ -927,13 +927,13 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A14" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="23"/>
       <c r="C14" s="23"/>
       <c r="D14" s="24">
         <f>MIN(1,D12/D7)</f>
-        <v>0.87951599999999996</v>
+        <v>0.98546</v>
       </c>
       <c r="E14" s="20"/>
       <c r="F14" s="22"/>
@@ -952,7 +952,7 @@
     </row>
     <row r="16" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A16" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="25"/>
       <c r="C16" s="25"/>
@@ -964,16 +964,16 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A17" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="C17" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="D17" s="27" t="s">
         <v>20</v>
-      </c>
-      <c r="D17" s="27" t="s">
-        <v>21</v>
       </c>
       <c r="E17" s="20"/>
       <c r="F17" s="22"/>
@@ -982,7 +982,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A18" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="28">
         <v>161.38</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A19" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="28">
         <v>53.79</v>
@@ -1022,7 +1022,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A20" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="29"/>
       <c r="C20" s="45"/>
@@ -1047,7 +1047,7 @@
     </row>
     <row r="22" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A22" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22" s="25"/>
       <c r="C22" s="25"/>
@@ -1059,19 +1059,19 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A23" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="C23" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="27" t="s">
+      <c r="D23" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="27" t="s">
         <v>28</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>29</v>
       </c>
       <c r="F23" s="22"/>
       <c r="G23" s="22"/>
@@ -1079,20 +1079,20 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A24" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="21">
-        <v>85</v>
+        <v>299</v>
       </c>
       <c r="C24" s="21">
-        <v>85</v>
+        <v>200</v>
       </c>
       <c r="D24" s="41">
         <v>2147483647</v>
       </c>
       <c r="E24" s="42">
         <f>C24*D24</f>
-        <v>182536109995</v>
+        <v>429496729400</v>
       </c>
       <c r="F24" s="22"/>
       <c r="G24" s="22"/>
@@ -1100,20 +1100,20 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A25" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="21">
         <v>17164</v>
       </c>
       <c r="C25" s="21">
-        <v>17164</v>
+        <v>0</v>
       </c>
       <c r="D25" s="41">
         <v>4000000</v>
       </c>
       <c r="E25" s="42">
         <f>C25*D25</f>
-        <v>68656000000</v>
+        <v>0</v>
       </c>
       <c r="F25" s="22"/>
       <c r="G25" s="22"/>
@@ -1121,20 +1121,20 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A26" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="21">
         <v>10000</v>
       </c>
       <c r="C26" s="21">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="D26" s="41">
         <v>1500000</v>
       </c>
       <c r="E26" s="42">
         <f>C26*D26</f>
-        <v>15000000000</v>
+        <v>0</v>
       </c>
       <c r="F26" s="22"/>
       <c r="G26" s="22"/>
@@ -1142,20 +1142,20 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A27" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="21">
         <v>15000</v>
       </c>
       <c r="C27" s="21">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="D27" s="41">
         <v>200000</v>
       </c>
       <c r="E27" s="42">
         <f>C27*D27</f>
-        <v>3000000000</v>
+        <v>0</v>
       </c>
       <c r="F27" s="22"/>
       <c r="G27" s="22"/>
@@ -1163,20 +1163,20 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A28" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" s="21">
         <v>30000</v>
       </c>
       <c r="C28" s="21">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="D28" s="41">
         <v>100000</v>
       </c>
       <c r="E28" s="42">
         <f>C28*D28</f>
-        <v>3000000000</v>
+        <v>0</v>
       </c>
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
@@ -1184,14 +1184,14 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A29" s="33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
       <c r="D29" s="43"/>
       <c r="E29" s="43">
         <f>SUM(E24:E28)</f>
-        <v>272192109995</v>
+        <v>429496729400</v>
       </c>
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
@@ -1199,14 +1199,14 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A30" s="14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" s="23"/>
       <c r="C30" s="23"/>
       <c r="D30" s="44"/>
       <c r="E30" s="44">
         <f>MAX(0,$D$13-E29)</f>
-        <v>330227890005</v>
+        <v>0</v>
       </c>
       <c r="F30" s="22"/>
       <c r="G30" s="22"/>
@@ -1214,14 +1214,14 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A31" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B31" s="30"/>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
       <c r="E31" s="24">
         <f>MIN(1,($D$12+E29)/$D$7)</f>
-        <v>0.93395442199900003</v>
+        <v>1</v>
       </c>
       <c r="F31" s="22"/>
       <c r="G31" s="22"/>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="33" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A33" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B33" s="31"/>
       <c r="C33" s="31"/>
@@ -1251,33 +1251,33 @@
     </row>
     <row r="34" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A34" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="32" t="s">
+      <c r="C34" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="32" t="s">
+      <c r="D34" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="32" t="s">
+      <c r="E34" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="E34" s="32" t="s">
+      <c r="F34" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="F34" s="32" t="s">
+      <c r="G34" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="G34" s="32" t="s">
+      <c r="H34" s="32" t="s">
         <v>45</v>
-      </c>
-      <c r="H34" s="32" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A35" s="35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="46">
         <v>13784000</v>
@@ -1299,16 +1299,16 @@
       </c>
       <c r="G35" s="37">
         <f>$D$13/F35</f>
-        <v>4.3783420292730622</v>
+        <v>0.52837798467539532</v>
       </c>
       <c r="H35" s="37">
         <f>$E$30/F35</f>
-        <v>2.4000707978603852</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A36" s="38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="47">
         <v>17409000</v>
@@ -1330,11 +1330,11 @@
       </c>
       <c r="G36" s="40">
         <f>$D$13/F36</f>
-        <v>3.8316023339727381</v>
+        <v>0.46239747963184835</v>
       </c>
       <c r="H36" s="40">
         <f>$E$30/F36</f>
-        <v>2.1003651175028231</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.5">
@@ -1349,7 +1349,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A38" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -1361,7 +1361,7 @@
     </row>
     <row r="39" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A39" s="52" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B39" s="53"/>
       <c r="C39" s="53"/>
@@ -1373,7 +1373,7 @@
     </row>
     <row r="40" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A40" s="52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B40" s="53"/>
       <c r="C40" s="53"/>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="41" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A41" s="52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B41" s="53"/>
       <c r="C41" s="53"/>

</xml_diff>